<commit_message>
Removed a lot of the testcases. Only added three in total. One negative for is RELMIDS is present an no TM is present and two positive. One for RELMIDS and TM is present and one for none are present
</commit_message>
<xml_diff>
--- a/rules/CORE-000777/negative/01/data/unit-test-coreid-CG0502-negative.xlsx
+++ b/rules/CORE-000777/negative/01/data/unit-test-coreid-CG0502-negative.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,6 +572,62 @@
       <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>$RELMIDS_EXISTS</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -632,7 +688,7 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>MIDS</t>
+          <t>RELMIDS</t>
         </is>
       </c>
     </row>
@@ -679,8 +735,7 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Disease Milestone
-Instance Name</t>
+          <t>Relationship to Disease Milestone Instance Name</t>
         </is>
       </c>
     </row>
@@ -757,7 +812,7 @@
         <v>8</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -801,7 +856,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>DIAG</t>
+          <t>AT TIME OF</t>
         </is>
       </c>
     </row>
@@ -846,7 +901,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>DIAG</t>
+          <t>AFTER</t>
         </is>
       </c>
     </row>

</xml_diff>